<commit_message>
docs: documentos actualizados a mysql y modelos en mysql workbench
</commit_message>
<xml_diff>
--- a/documentos/fase1/07_Diccionario_de_Datos.xlsx
+++ b/documentos/fase1/07_Diccionario_de_Datos.xlsx
@@ -1363,7 +1363,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -1418,7 +1418,7 @@
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>REGEXP_LIKE(codigo_dane, '^[0-9]{2}$')</t>
+          <t>codigo_dane REGEXP '^[0-9]{2}$'</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(60)</t>
+          <t>VARCHAR(60)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1539,7 +1539,7 @@
       <c r="F6" s="3" t="inlineStr"/>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>REGEXP_LIKE(codigo_dane, '^[0-9]{5}$')</t>
+          <t>codigo_dane REGEXP '^[0-9]{5}$'</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(80)</t>
+          <t>VARCHAR(80)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(80)</t>
+          <t>VARCHAR(80)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(120)</t>
+          <t>VARCHAR(120)</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(20)</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(100)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(3)</t>
+          <t>VARCHAR(3)</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(15)</t>
+          <t>VARCHAR(15)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(60)</t>
+          <t>VARCHAR(60)</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(60)</t>
+          <t>VARCHAR(60)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(20)</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(100)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(12,2)</t>
+          <t>DECIMAL(12,2)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(10)</t>
+          <t>VARCHAR(10)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(20)</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(100)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(20)</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(100)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(10)</t>
+          <t>VARCHAR(10)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(60)</t>
+          <t>VARCHAR(60)</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(200)</t>
+          <t>VARCHAR(200)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(8)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(3)</t>
+          <t>VARCHAR(3)</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(15)</t>
+          <t>VARCHAR(15)</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(60)</t>
+          <t>VARCHAR(60)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(60)</t>
+          <t>VARCHAR(60)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(100)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(120)</t>
+          <t>VARCHAR(120)</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -3284,7 +3284,7 @@
       <c r="E52" s="3" t="inlineStr"/>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>SYSDATE</t>
+          <t>CURRENT_TIMESTAMP</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr"/>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(8)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(20)</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -3390,7 +3390,7 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(10)</t>
+          <t>VARCHAR(10)</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(3)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(40)</t>
+          <t>VARCHAR(40)</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(5)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(60)</t>
+          <t>VARCHAR(60)</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(10)</t>
+          <t>VARCHAR(10)</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(3)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(8)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(40)</t>
+          <t>VARCHAR(40)</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(40)</t>
+          <t>VARCHAR(40)</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(15)</t>
+          <t>VARCHAR(15)</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(10)</t>
+          <t>VARCHAR(10)</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(5)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(8)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -4060,7 +4060,7 @@
       <c r="E72" s="3" t="inlineStr"/>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>SYSDATE</t>
+          <t>CURRENT_TIMESTAMP</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr"/>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(8)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(12)</t>
+          <t>VARCHAR(12)</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(8)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(10)</t>
+          <t>VARCHAR(10)</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(200)</t>
+          <t>VARCHAR(200)</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(200)</t>
+          <t>VARCHAR(200)</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -4345,7 +4345,7 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(400)</t>
+          <t>VARCHAR(400)</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -4380,7 +4380,7 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(10)</t>
+          <t>VARCHAR(10)</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(80)</t>
+          <t>VARCHAR(80)</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -4497,7 +4497,7 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(20)</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(10,2)</t>
+          <t>DECIMAL(10,2)</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(10)</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -4670,7 +4670,7 @@
       <c r="G88" s="3" t="inlineStr"/>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>Fecha y hora programada (DATE de Oracle guarda la hora).</t>
+          <t>Fecha y hora programada de la cita.</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(200)</t>
+          <t>VARCHAR(200)</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(12)</t>
+          <t>VARCHAR(12)</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(8)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -4848,7 +4848,7 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -4887,7 +4887,7 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
@@ -4926,7 +4926,7 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(10)</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -4965,7 +4965,7 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(10)</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
@@ -5004,7 +5004,7 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -5078,7 +5078,7 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(5,2)</t>
+          <t>DECIMAL(5,2)</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4,1)</t>
+          <t>DECIMAL(4,1)</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
@@ -5156,7 +5156,7 @@
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(3)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
@@ -5195,7 +5195,7 @@
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(400)</t>
+          <t>VARCHAR(400)</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(400)</t>
+          <t>VARCHAR(400)</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(400)</t>
+          <t>VARCHAR(400)</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(12)</t>
+          <t>VARCHAR(12)</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
@@ -5378,7 +5378,7 @@
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(80)</t>
+          <t>VARCHAR(80)</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
@@ -5417,7 +5417,7 @@
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(80)</t>
+          <t>VARCHAR(80)</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(40)</t>
+          <t>VARCHAR(40)</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
@@ -5491,7 +5491,7 @@
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(60)</t>
+          <t>VARCHAR(60)</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
@@ -5526,7 +5526,7 @@
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(10,2)</t>
+          <t>DECIMAL(10,2)</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(10)</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(60)</t>
+          <t>VARCHAR(60)</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(3)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
@@ -5760,7 +5760,7 @@
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(3)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
@@ -5838,7 +5838,7 @@
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(200)</t>
+          <t>VARCHAR(200)</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
@@ -5912,7 +5912,7 @@
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
@@ -5990,7 +5990,7 @@
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
@@ -6029,7 +6029,7 @@
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
@@ -6040,7 +6040,7 @@
       <c r="E124" s="3" t="inlineStr"/>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>SYSDATE</t>
+          <t>CURRENT_TIMESTAMP</t>
         </is>
       </c>
       <c r="G124" s="3" t="inlineStr"/>
@@ -6068,7 +6068,7 @@
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(10)</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(15)</t>
+          <t>VARCHAR(15)</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
@@ -6181,7 +6181,7 @@
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(16)</t>
+          <t>VARCHAR(16)</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
@@ -6220,7 +6220,7 @@
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>VARCHAR2(10)</t>
+          <t>VARCHAR(10)</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(8)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
@@ -6302,7 +6302,7 @@
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
@@ -6341,7 +6341,7 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
@@ -6380,7 +6380,7 @@
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(10)</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(3)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
@@ -6462,7 +6462,7 @@
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(4)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
@@ -6501,7 +6501,7 @@
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(6)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
@@ -6536,7 +6536,7 @@
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(5)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
@@ -6575,7 +6575,7 @@
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(10,2)</t>
+          <t>DECIMAL(10,2)</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>NUMBER(5,2)</t>
+          <t>DECIMAL(5,2)</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: correcciones y tono natural en los documentos Word
Errores corregidos: regex del diccionario convertida en nota al pie, script 02_comentarios.sql que no existe, limites de Oracle Free en los supuestos, MINUS en vez de EXCEPT, VET_APP, ejercicio 22 en vez de 21, rutas entregables/ y docs/src, paginacion que la app no tiene. Frases telegraficas reescritas sin pasar del 5 % de palabras por documento. El diccionario .xlsx y el DDL de Workbench pasan a relaciones en infinitivo.
</commit_message>
<xml_diff>
--- a/documentos/fase1/07_Diccionario_de_Datos.xlsx
+++ b/documentos/fase1/07_Diccionario_de_Datos.xlsx
@@ -811,7 +811,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Resuelve la relación N:M CERTIFICADO_EN entre VETERINARIO y ESPECIALIDAD.</t>
+          <t>Resuelve la relación N:M CERTIFICAR entre VETERINARIO y ESPECIALIDAD.</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Historia clínica única de cada mascota (relación 1:1 TIENE), compartida por todas las sedes.</t>
+          <t>Historia clínica única de cada mascota (relación 1:1 TENER), compartida por todas las sedes.</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Registro clínico de una cita atendida (relación 1:1 GENERA con CITA).</t>
+          <t>Registro clínico de una cita atendida (relación 1:1 GENERAR con CITA).</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Resuelve la relación N:M PRESCRIBE entre CONSULTA y MEDICAMENTO (fórmula médica).</t>
+          <t>Resuelve la relación N:M PRESCRIBIR entre CONSULTA y MEDICAMENTO (fórmula médica).</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Resuelve la relación N:M ALMACENA entre SEDE y MEDICAMENTO: existencias por sede.</t>
+          <t>Resuelve la relación N:M ALMACENAR entre SEDE y MEDICAMENTO: existencias por sede.</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1922,7 @@
       <c r="G16" s="3" t="inlineStr"/>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Empleado que dirige la sede (relación 1:1 DIRIGE).</t>
+          <t>Empleado que dirige la sede (relación 1:1 DIRIGIR).</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -2417,7 +2417,7 @@
       <c r="G29" s="3" t="inlineStr"/>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Sede donde labora el empleado (relación LABORA_EN).</t>
+          <t>Sede donde labora el empleado (relación LABORAR).</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -6722,7 +6722,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>PERTENECE_A</t>
+          <t>PERTENECER</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -6754,7 +6754,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>UBICADA_EN</t>
+          <t>UBICAR</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -6786,7 +6786,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>DIRIGE</t>
+          <t>DIRIGIR</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>LABORA_EN</t>
+          <t>LABORAR</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -6850,7 +6850,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>ES_UN</t>
+          <t>EJERCER</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -6882,7 +6882,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>ES_UN</t>
+          <t>COLABORAR</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>CERTIFICADO_EN</t>
+          <t>CERTIFICAR</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -6946,7 +6946,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>CERTIFICADO_EN</t>
+          <t>CERTIFICAR</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -6978,7 +6978,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>RESIDE_EN</t>
+          <t>RESIDIR</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -7010,7 +7010,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>TIENE_TELEFONO</t>
+          <t>REGISTRAR</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -7042,7 +7042,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>CLASIFICA</t>
+          <t>AGRUPAR</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>ES_DE_RAZA</t>
+          <t>CLASIFICAR</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>PROPIETARIO_DE</t>
+          <t>POSEER</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -7138,7 +7138,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>TIENE</t>
+          <t>TENER</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>SOLICITA</t>
+          <t>SOLICITAR</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>ATIENDE</t>
+          <t>ATENDER</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>SE_PROGRAMA_EN</t>
+          <t>PROGRAMAR</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -7266,7 +7266,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>CORRESPONDE_A</t>
+          <t>CORRESPONDER</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>GENERA</t>
+          <t>GENERAR</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>ASISTE</t>
+          <t>ASISTIR</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -7362,7 +7362,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>PRESCRIBE</t>
+          <t>PRESCRIBIR</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>PRESCRIBE</t>
+          <t>PRESCRIBIR</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -7426,7 +7426,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>ALMACENA</t>
+          <t>ALMACENAR</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>ALMACENA</t>
+          <t>ALMACENAR</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>FACTURADA_A</t>
+          <t>FACTURAR</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>EMITIDA_EN</t>
+          <t>EXPEDIR</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -7554,7 +7554,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>EMITE</t>
+          <t>EMITIR</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>CONTIENE</t>
+          <t>CONTENER</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -7618,7 +7618,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>INCLUYE_SERVICIO</t>
+          <t>COBRAR</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -7650,7 +7650,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>INCLUYE_MEDICAMENTO</t>
+          <t>VENDER</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: revision completa de base de datos, app y documentos; presentacion nueva en PowerPoint
Se probaron la base y la app, se corrigieron los documentos, los README y los nombres de relacion,
las claves de cargar_bd.sh ya no viajan en la linea de comandos, y se reemplazan las versiones
viejas del documento final y de la presentacion.
</commit_message>
<xml_diff>
--- a/documentos/fase1/07_Diccionario_de_Datos.xlsx
+++ b/documentos/fase1/07_Diccionario_de_Datos.xlsx
@@ -811,7 +811,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Resuelve la relación N:M CERTIFICADO_EN entre VETERINARIO y ESPECIALIDAD.</t>
+          <t>Resuelve la relación N:M CERTIFICAR entre VETERINARIO y ESPECIALIDAD.</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Historia clínica única de cada mascota (relación 1:1 TIENE), compartida por todas las sedes.</t>
+          <t>Historia clínica única de cada mascota (relación 1:1 TENER), compartida por todas las sedes.</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Registro clínico de una cita atendida (relación 1:1 GENERA con CITA).</t>
+          <t>Registro clínico de una cita atendida (relación 1:1 GENERAR con CITA).</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Resuelve la relación N:M PRESCRIBE entre CONSULTA y MEDICAMENTO (fórmula médica).</t>
+          <t>Resuelve la relación N:M PRESCRIBIR entre CONSULTA y MEDICAMENTO (fórmula médica).</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Resuelve la relación N:M ALMACENA entre SEDE y MEDICAMENTO: existencias por sede.</t>
+          <t>Resuelve la relación N:M ALMACENAR entre SEDE y MEDICAMENTO: existencias por sede.</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1922,7 @@
       <c r="G16" s="3" t="inlineStr"/>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Empleado que dirige la sede (relación 1:1 DIRIGE).</t>
+          <t>Empleado que dirige la sede (relación 1:1 DIRIGIR).</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -2417,7 +2417,7 @@
       <c r="G29" s="3" t="inlineStr"/>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Sede donde labora el empleado (relación LABORA_EN).</t>
+          <t>Sede donde labora el empleado (relación LABORAR).</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -6722,7 +6722,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>PERTENECE_A</t>
+          <t>PERTENECER</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -6754,7 +6754,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>UBICADA_EN</t>
+          <t>UBICAR</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -6786,7 +6786,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>DIRIGE</t>
+          <t>DIRIGIR</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>LABORA_EN</t>
+          <t>LABORAR</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -6850,7 +6850,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>ES_UN</t>
+          <t>EJERCER</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -6882,7 +6882,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>ES_UN</t>
+          <t>COLABORAR</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>CERTIFICADO_EN</t>
+          <t>CERTIFICAR</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -6946,7 +6946,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>CERTIFICADO_EN</t>
+          <t>CERTIFICAR</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -6978,7 +6978,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>RESIDE_EN</t>
+          <t>RESIDIR</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -7010,7 +7010,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>TIENE_TELEFONO</t>
+          <t>REGISTRAR</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -7042,7 +7042,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>CLASIFICA</t>
+          <t>AGRUPAR</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>ES_DE_RAZA</t>
+          <t>CLASIFICAR</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>PROPIETARIO_DE</t>
+          <t>POSEER</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -7138,7 +7138,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>TIENE</t>
+          <t>TENER</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>SOLICITA</t>
+          <t>SOLICITAR</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>ATIENDE</t>
+          <t>ATENDER</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>SE_PROGRAMA_EN</t>
+          <t>PROGRAMAR</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -7266,7 +7266,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>CORRESPONDE_A</t>
+          <t>CORRESPONDER</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>GENERA</t>
+          <t>GENERAR</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>ASISTE</t>
+          <t>ASISTIR</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -7362,7 +7362,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>PRESCRIBE</t>
+          <t>PRESCRIBIR</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>PRESCRIBE</t>
+          <t>PRESCRIBIR</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -7426,7 +7426,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>ALMACENA</t>
+          <t>ALMACENAR</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>ALMACENA</t>
+          <t>ALMACENAR</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>FACTURADA_A</t>
+          <t>FACTURAR</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>EMITIDA_EN</t>
+          <t>EXPEDIR</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -7554,7 +7554,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>EMITE</t>
+          <t>EMITIR</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>CONTIENE</t>
+          <t>CONTENER</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -7618,7 +7618,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>INCLUYE_SERVICIO</t>
+          <t>COBRAR</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -7650,7 +7650,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>INCLUYE_MEDICAMENTO</t>
+          <t>VENDER</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">

</xml_diff>